<commit_message>
Remove do painel 4 colaboradoras demitidas
Amanda de Araujo Santos, Camilla Emanuelle Lopes de Almeida, Joanna Roberta
de Queiroz Viana e Juliene Reis Ferreira entram em EXCLUDED_NAMES e saem do
mapa de gestores. Os avisos por gestor eram so sobre elas e ficam zerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -497,210 +497,210 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B13" t="str">
-        <v>Camilla Emanuelle Lopes de Almeida</v>
+        <v>Camille Kauane Da Silva Nunes</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B14" t="str">
-        <v>Camille Kauane Da Silva Nunes</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B15" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Claudio Bispo Dos Santos</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B16" t="str">
-        <v>Claudio Bispo Dos Santos</v>
+        <v>Danielle Dos Santos Silva</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B17" t="str">
-        <v>Danielle Dos Santos Silva</v>
+        <v>Danrley firmino dos santos</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B18" t="str">
-        <v>Danrley firmino dos santos</v>
+        <v>Deise Gislaine Silva vitor</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B19" t="str">
-        <v>Deise Gislaine Silva vitor</v>
+        <v>Edna Lopes Da Silva</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B20" t="str">
-        <v>Edna Lopes Da Silva</v>
+        <v>Eduarda Pereira Costa Silva</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B21" t="str">
-        <v>Eduarda Pereira Costa Silva</v>
+        <v>Eliene Da Silva Santos</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B22" t="str">
-        <v>Eliene Da Silva Santos</v>
+        <v>Emanoelle Feitosa Vieira Santos</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B23" t="str">
-        <v>Emanoelle Feitosa Vieira Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B24" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Fabia Batista da Silva</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B25" t="str">
-        <v>Fabia Batista da Silva</v>
+        <v>Gessica Aparecida Dos Santos</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B26" t="str">
-        <v>Gessica Aparecida Dos Santos</v>
+        <v>Gessyca Nayara Rocha Santos</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B27" t="str">
-        <v>Gessyca Nayara Rocha Santos</v>
+        <v>Giselle Dos Santos Roberto</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B28" t="str">
-        <v>Giselle Dos Santos Roberto</v>
+        <v>Hugo Castro Lopes</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B29" t="str">
-        <v>Hugo Castro Lopes</v>
+        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v>Romulo Jose Santos Lisboa</v>
+      </c>
+      <c r="B30" t="str">
         <v>Joao Antonio Tavares Santos</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B31" t="str">
-        <v>Joanna Roberta de Queiroz Viana</v>
+        <v>João Ricardo Dantas Albuquerque</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B32" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>João Victor Santos da Silva</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B33" t="str">
-        <v>João Ricardo Dantas Albuquerque</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B34" t="str">
-        <v>João Victor Santos da Silva</v>
+        <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B35" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Josimara Ferreira Monteiro</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B36" t="str">
-        <v>Jordelle Meygre Costa De Oliveira</v>
+        <v>Juliene bezerra</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B37" t="str">
-        <v>Josimara Ferreira Monteiro</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B38" t="str">
-        <v>Juliene bezerra</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
     </row>
     <row r="39">
@@ -708,15 +708,15 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B39" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B40" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Lays da Silva Vieira</v>
       </c>
     </row>
     <row r="41">
@@ -724,47 +724,47 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B41" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Leticia Seixas Santos</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B42" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Letícia Soares Belo</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B43" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B44" t="str">
-        <v>Letícia Soares Belo</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B45" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Luciano Torres</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B46" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Ludmylla Wolpert Melo</v>
       </c>
     </row>
     <row r="47">
@@ -772,7 +772,7 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B47" t="str">
-        <v>Luciano Torres</v>
+        <v>Luiz Fellipe Guedes Santos Silva</v>
       </c>
     </row>
     <row r="48">
@@ -780,127 +780,127 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B48" t="str">
-        <v>Ludmylla Wolpert Melo</v>
+        <v>Marcio Alif Santos Silva</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="B49" t="str">
-        <v>Luiz Fellipe Guedes Santos Silva</v>
+        <v>Mariane Santos Sousa</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B50" t="str">
-        <v>Marcio Alif Santos Silva</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Leidiane Souza</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B51" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B52" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B53" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Maria Nobre Farias De França</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B54" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B55" t="str">
-        <v>Maria Nobre Farias De França</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B56" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B57" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B58" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Paulo Cesar Da Silva Santos Junior</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B59" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Pedro Lucas Rocha da Fonseca</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B60" t="str">
-        <v>Paulo Cesar Da Silva Santos Junior</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B61" t="str">
-        <v>Pedro Lucas Rocha da Fonseca</v>
+        <v>Ravy Thiago Vieira Da Silva</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B62" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Robéria Gilo Da Silva</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B63" t="str">
-        <v>Ravy Thiago Vieira Da Silva</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
     </row>
     <row r="64">
@@ -908,23 +908,23 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B64" t="str">
-        <v>Robéria Gilo Da Silva</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Sem Gestor</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B65" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B66" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
     </row>
     <row r="67">
@@ -932,87 +932,87 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B67" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B68" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Thalys Gomes Dos Santos</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B69" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B70" t="str">
-        <v>Thalys Gomes Dos Santos</v>
+        <v>Thayane Mayara dos Santos</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B71" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B72" t="str">
-        <v>Thayane Mayara dos Santos</v>
+        <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B73" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B74" t="str">
-        <v>Valesca Meirelle Bezerra Vitória</v>
+        <v>Yasmin Abilia Ferro da Silva</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B75" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Yuri Castro Gomes</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B76" t="str">
-        <v>Yasmin Abilia Ferro da Silva</v>
+        <v>Josenildo Alves da silva Júnior</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B77" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Shayane Oliveira Ferreira</v>
       </c>
     </row>
     <row r="78">
@@ -1020,15 +1020,15 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B78" t="str">
-        <v>Josenildo Alves da silva Júnior</v>
+        <v>Maria Fernanda Gomes Vieira</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B79" t="str">
-        <v>Shayane Oliveira Ferreira</v>
+        <v>Nayara Soares Kimura</v>
       </c>
     </row>
     <row r="80">
@@ -1036,31 +1036,31 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B80" t="str">
-        <v>Maria Fernanda Gomes Vieira</v>
+        <v>Caroline leite dos santos</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B81" t="str">
-        <v>Nayara Soares Kimura</v>
+        <v>Rayanne Ferreira</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B82" t="str">
-        <v>Caroline leite dos santos</v>
+        <v>Luciene Tayná Félix da Silva</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B83" t="str">
-        <v>Rayanne Ferreira</v>
+        <v>Bruna Soares Siqueira</v>
       </c>
     </row>
     <row r="84">
@@ -1068,23 +1068,23 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B84" t="str">
-        <v>Luciene Tayná Félix da Silva</v>
+        <v>Edlane Silva de Lima</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B85" t="str">
-        <v>Bruna Soares Siqueira</v>
+        <v>Jayane da Silva Dias</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B86" t="str">
-        <v>Edlane Silva de Lima</v>
+        <v>Rayanne Maria dos Santos Moca</v>
       </c>
     </row>
     <row r="87">
@@ -1092,124 +1092,92 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B87" t="str">
-        <v>Jayane da Silva Dias</v>
+        <v>Evellyn Vitória Nunes Santos</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B88" t="str">
-        <v>Rayanne Maria dos Santos Moca</v>
+        <v>Samuel Monteiro da Silva</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B89" t="str">
-        <v>Evellyn Vitória Nunes Santos</v>
+        <v>Juliana Francine Marques da Silva</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B90" t="str">
-        <v>Samuel Monteiro da Silva</v>
+        <v>Tayna Monaisa Vasconcelos santos</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B91" t="str">
-        <v>Juliana Francine Marques da Silva</v>
+        <v>Auda da Conceição Santos</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B92" t="str">
-        <v>Juliene Reis Ferreira</v>
+        <v>Sione Barbosa da Silva</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B93" t="str">
-        <v>Tayna Monaisa Vasconcelos santos</v>
+        <v>Sabrina Barbosa Machado Mariano</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B94" t="str">
-        <v>Amanda de Araújo Santos</v>
+        <v>João Paulo Vieira Melo</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B95" t="str">
-        <v>Auda da Conceição Santos</v>
+        <v>Crislaine Freire dos Santos</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B96" t="str">
-        <v>Sione Barbosa da Silva</v>
+        <v>Kledja Nunes da Silva</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B97" t="str">
-        <v>Sabrina Barbosa Machado Mariano</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B98" t="str">
-        <v>João Paulo Vieira Melo</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>Joao Antonio Tavares Santos</v>
-      </c>
-      <c r="B99" t="str">
-        <v>Crislaine Freire dos Santos</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>Joao Antonio Tavares Santos</v>
-      </c>
-      <c r="B100" t="str">
-        <v>Kledja Nunes da Silva</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>Tomás Azevedo Santos</v>
-      </c>
-      <c r="B101" t="str">
         <v>Luís Henrique Batista dos Santos</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B97"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reorganiza equipes de Taciane, Kemilly e Mariane e cria acesso da Keliany
- Mariane: Deise, Maria Fernanda e Anny Karoline (vindas da Taciane)
- Keliany Cordeiro (novo acesso no codigo 1010, sem mes de aniversario):
  Edlane, Maria Cicilia, Yasmin Abilia, Bruna Soares, Eduarda e Luciene
  Tayna (vindas da Kemilly)
- Kemilly: fica com Maryanna e Nayara e recebe o resto da equipe da
  Taciane, que fica sem colaboradores
- Remove a linha "Rayanne Ferreira" do mapa: era a Rayanne Maria dos
  Santos Moca cadastrada com nome curto

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Saldos_por_Gestor_Ajustado.xlsx
+++ b/public/Saldos_por_Gestor_Ajustado.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B97"/>
+  <dimension ref="A1:B96"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -441,7 +441,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B6" t="str">
         <v>Ana Paula Amaral Santos Ismerim</v>
@@ -457,7 +457,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B8" t="str">
         <v>Anny Karoline Andrade Santos</v>
@@ -473,7 +473,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B10" t="str">
         <v>Bruna Rayane Oliveira dos Santos</v>
@@ -497,7 +497,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B13" t="str">
         <v>Camille Kauane Da Silva Nunes</v>
@@ -537,7 +537,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B18" t="str">
         <v>Deise Gislaine Silva vitor</v>
@@ -553,7 +553,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B20" t="str">
         <v>Eduarda Pereira Costa Silva</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B21" t="str">
         <v>Eliene Da Silva Santos</v>
@@ -801,7 +801,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B51" t="str">
         <v>Maria Cicília Brito Veiga</v>
@@ -985,7 +985,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B74" t="str">
         <v>Yasmin Abilia Ferro da Silva</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B76" t="str">
         <v>Josenildo Alves da silva Júnior</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B77" t="str">
         <v>Shayane Oliveira Ferreira</v>
@@ -1017,7 +1017,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B78" t="str">
         <v>Maria Fernanda Gomes Vieira</v>
@@ -1033,7 +1033,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B80" t="str">
         <v>Caroline leite dos santos</v>
@@ -1041,26 +1041,26 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B81" t="str">
-        <v>Rayanne Ferreira</v>
+        <v>Luciene Tayná Félix da Silva</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B82" t="str">
-        <v>Luciene Tayná Félix da Silva</v>
+        <v>Bruna Soares Siqueira</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Keliany Cordeiro</v>
       </c>
       <c r="B83" t="str">
-        <v>Bruna Soares Siqueira</v>
+        <v>Edlane Silva de Lima</v>
       </c>
     </row>
     <row r="84">
@@ -1068,47 +1068,47 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B84" t="str">
-        <v>Edlane Silva de Lima</v>
+        <v>Jayane da Silva Dias</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B85" t="str">
-        <v>Jayane da Silva Dias</v>
+        <v>Rayanne Maria dos Santos Moca</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B86" t="str">
-        <v>Rayanne Maria dos Santos Moca</v>
+        <v>Evellyn Vitória Nunes Santos</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B87" t="str">
-        <v>Evellyn Vitória Nunes Santos</v>
+        <v>Samuel Monteiro da Silva</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B88" t="str">
-        <v>Samuel Monteiro da Silva</v>
+        <v>Juliana Francine Marques da Silva</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B89" t="str">
-        <v>Juliana Francine Marques da Silva</v>
+        <v>Tayna Monaisa Vasconcelos santos</v>
       </c>
     </row>
     <row r="90">
@@ -1116,23 +1116,23 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B90" t="str">
-        <v>Tayna Monaisa Vasconcelos santos</v>
+        <v>Auda da Conceição Santos</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B91" t="str">
-        <v>Auda da Conceição Santos</v>
+        <v>Sione Barbosa da Silva</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B92" t="str">
-        <v>Sione Barbosa da Silva</v>
+        <v>Sabrina Barbosa Machado Mariano</v>
       </c>
     </row>
     <row r="93">
@@ -1140,15 +1140,15 @@
         <v>Suzana Martins Tavares</v>
       </c>
       <c r="B93" t="str">
-        <v>Sabrina Barbosa Machado Mariano</v>
+        <v>João Paulo Vieira Melo</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B94" t="str">
-        <v>João Paulo Vieira Melo</v>
+        <v>Crislaine Freire dos Santos</v>
       </c>
     </row>
     <row r="95">
@@ -1156,28 +1156,20 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B95" t="str">
-        <v>Crislaine Freire dos Santos</v>
+        <v>Kledja Nunes da Silva</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="B96" t="str">
-        <v>Kledja Nunes da Silva</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>Tomás Azevedo Santos</v>
-      </c>
-      <c r="B97" t="str">
         <v>Luís Henrique Batista dos Santos</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B96"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>